<commit_message>
Add actual price row and AMG Greek scaling
</commit_message>
<xml_diff>
--- a/templates/AMG_Excel.xlsx
+++ b/templates/AMG_Excel.xlsx
@@ -8,17 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\great\Downloads\AMG Models\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98FB009-E829-44FE-8044-7535E7F58D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6F97C44-6AB8-4DE6-911E-681051861CC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{47BAF088-3042-44C3-893B-F852E1C1EF9C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="18720" activeTab="1" xr2:uid="{47BAF088-3042-44C3-893B-F852E1C1EF9C}"/>
   </bookViews>
   <sheets>
     <sheet name="Input" sheetId="1" r:id="rId1"/>
     <sheet name="Output" sheetId="3" r:id="rId2"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId3"/>
-  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="47">
   <si>
     <t>Time (in years)</t>
   </si>
@@ -181,6 +178,9 @@
   </si>
   <si>
     <t>\</t>
+  </si>
+  <si>
+    <t>Actual Price</t>
   </si>
 </sst>
 </file>
@@ -189,9 +189,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="_(&quot;$&quot;* #,##0.0000_);_(&quot;$&quot;* \(#,##0.0000\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.0000_);_(&quot;$&quot;* \(#,##0.0000\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -597,6 +597,68 @@
   </cellStyleXfs>
   <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -624,68 +686,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="166" fontId="12" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="12" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="centerContinuous"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="10" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1539,446 +1539,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-      <xxl21:relativeUrl r:id="rId3"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="__FDSCACHE__"/>
-      <sheetName val="BSM"/>
-      <sheetName val="BSM '76"/>
-      <sheetName val="Payoff Diagram"/>
-      <sheetName val="Capital Allocation Slide"/>
-      <sheetName val="Control"/>
-      <sheetName val="DCF"/>
-      <sheetName val="Comps"/>
-      <sheetName val="DCF Output"/>
-      <sheetName val="Comps Output"/>
-      <sheetName val="Price Output"/>
-      <sheetName val="__APW_ACTIVE_FIELD_RESTORE__"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3">
-        <row r="9">
-          <cell r="J9">
-            <v>80</v>
-          </cell>
-          <cell r="O9">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="J10">
-            <v>81</v>
-          </cell>
-          <cell r="O10">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="J11">
-            <v>82</v>
-          </cell>
-          <cell r="O11">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="J12">
-            <v>83</v>
-          </cell>
-          <cell r="O12">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="J13">
-            <v>84</v>
-          </cell>
-          <cell r="O13">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="J14">
-            <v>85</v>
-          </cell>
-          <cell r="O14">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="J15">
-            <v>86</v>
-          </cell>
-          <cell r="O15">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="J16">
-            <v>87</v>
-          </cell>
-          <cell r="O16">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="J17">
-            <v>88</v>
-          </cell>
-          <cell r="O17">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="J18">
-            <v>89</v>
-          </cell>
-          <cell r="O18">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="J19">
-            <v>90</v>
-          </cell>
-          <cell r="O19">
-            <v>0</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="J20">
-            <v>91</v>
-          </cell>
-          <cell r="O20">
-            <v>10000</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="J21">
-            <v>92</v>
-          </cell>
-          <cell r="O21">
-            <v>20000</v>
-          </cell>
-        </row>
-        <row r="22">
-          <cell r="J22">
-            <v>93</v>
-          </cell>
-          <cell r="O22">
-            <v>30000</v>
-          </cell>
-        </row>
-        <row r="23">
-          <cell r="J23">
-            <v>94</v>
-          </cell>
-          <cell r="O23">
-            <v>40000</v>
-          </cell>
-        </row>
-        <row r="24">
-          <cell r="J24">
-            <v>95</v>
-          </cell>
-          <cell r="O24">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="25">
-          <cell r="J25">
-            <v>96</v>
-          </cell>
-          <cell r="O25">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="26">
-          <cell r="J26">
-            <v>97</v>
-          </cell>
-          <cell r="O26">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="27">
-          <cell r="J27">
-            <v>98</v>
-          </cell>
-          <cell r="O27">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="28">
-          <cell r="J28">
-            <v>99</v>
-          </cell>
-          <cell r="O28">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="29">
-          <cell r="J29">
-            <v>100</v>
-          </cell>
-          <cell r="O29">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="30">
-          <cell r="J30">
-            <v>101</v>
-          </cell>
-          <cell r="O30">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="31">
-          <cell r="J31">
-            <v>102</v>
-          </cell>
-          <cell r="O31">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="32">
-          <cell r="J32">
-            <v>103</v>
-          </cell>
-          <cell r="O32">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="33">
-          <cell r="J33">
-            <v>104</v>
-          </cell>
-          <cell r="O33">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="34">
-          <cell r="J34">
-            <v>105</v>
-          </cell>
-          <cell r="O34">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="35">
-          <cell r="J35">
-            <v>106</v>
-          </cell>
-          <cell r="O35">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="36">
-          <cell r="J36">
-            <v>107</v>
-          </cell>
-          <cell r="O36">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="37">
-          <cell r="J37">
-            <v>108</v>
-          </cell>
-          <cell r="O37">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="38">
-          <cell r="J38">
-            <v>109</v>
-          </cell>
-          <cell r="O38">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="39">
-          <cell r="J39">
-            <v>110</v>
-          </cell>
-          <cell r="O39">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="40">
-          <cell r="J40">
-            <v>111</v>
-          </cell>
-          <cell r="O40">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="41">
-          <cell r="J41">
-            <v>112</v>
-          </cell>
-          <cell r="O41">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="42">
-          <cell r="J42">
-            <v>113</v>
-          </cell>
-          <cell r="O42">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="43">
-          <cell r="J43">
-            <v>114</v>
-          </cell>
-          <cell r="O43">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="44">
-          <cell r="J44">
-            <v>115</v>
-          </cell>
-          <cell r="O44">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="45">
-          <cell r="J45">
-            <v>116</v>
-          </cell>
-          <cell r="O45">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="46">
-          <cell r="J46">
-            <v>117</v>
-          </cell>
-          <cell r="O46">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="47">
-          <cell r="J47">
-            <v>118</v>
-          </cell>
-          <cell r="O47">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="48">
-          <cell r="J48">
-            <v>119</v>
-          </cell>
-          <cell r="O48">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="49">
-          <cell r="J49">
-            <v>120</v>
-          </cell>
-          <cell r="O49">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="50">
-          <cell r="J50">
-            <v>121</v>
-          </cell>
-          <cell r="O50">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="51">
-          <cell r="J51">
-            <v>122</v>
-          </cell>
-          <cell r="O51">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="52">
-          <cell r="J52">
-            <v>123</v>
-          </cell>
-          <cell r="O52">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="53">
-          <cell r="J53">
-            <v>124</v>
-          </cell>
-          <cell r="O53">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="54">
-          <cell r="J54">
-            <v>125</v>
-          </cell>
-          <cell r="O54">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="55">
-          <cell r="J55">
-            <v>126</v>
-          </cell>
-          <cell r="O55">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="56">
-          <cell r="J56">
-            <v>127</v>
-          </cell>
-          <cell r="O56">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="57">
-          <cell r="J57">
-            <v>128</v>
-          </cell>
-          <cell r="O57">
-            <v>50000</v>
-          </cell>
-        </row>
-        <row r="58">
-          <cell r="J58">
-            <v>129</v>
-          </cell>
-          <cell r="O58">
-            <v>50000</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2316,310 +1876,310 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="3"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="43"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-      <c r="M2" s="5"/>
-      <c r="N2" s="5"/>
-      <c r="O2" s="6"/>
+      <c r="A2" s="44"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="46"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="6"/>
+      <c r="A3" s="44"/>
+      <c r="B3" s="45"/>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45"/>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45"/>
+      <c r="I3" s="45"/>
+      <c r="J3" s="45"/>
+      <c r="K3" s="45"/>
+      <c r="L3" s="45"/>
+      <c r="M3" s="45"/>
+      <c r="N3" s="45"/>
+      <c r="O3" s="46"/>
     </row>
     <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
-      <c r="H4" s="8"/>
-      <c r="I4" s="8"/>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="9"/>
+      <c r="A4" s="47"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="48"/>
+      <c r="D4" s="48"/>
+      <c r="E4" s="48"/>
+      <c r="F4" s="48"/>
+      <c r="G4" s="48"/>
+      <c r="H4" s="48"/>
+      <c r="I4" s="48"/>
+      <c r="J4" s="48"/>
+      <c r="K4" s="48"/>
+      <c r="L4" s="48"/>
+      <c r="M4" s="48"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="49"/>
     </row>
     <row r="7" spans="1:15" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="49"/>
+      <c r="B7" s="39"/>
     </row>
     <row r="8" spans="1:15" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="49"/>
+      <c r="B8" s="39"/>
     </row>
     <row r="9" spans="1:15" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="49"/>
+      <c r="B9" s="39"/>
     </row>
     <row r="10" spans="1:15" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="49"/>
+      <c r="B10" s="39"/>
     </row>
     <row r="12" spans="1:15" ht="33" x14ac:dyDescent="0.45">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="14" t="s">
+      <c r="D12" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="G12" s="14" t="s">
+      <c r="G12" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="J12" s="14" t="s">
+      <c r="J12" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="11" t="s">
+      <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="44"/>
-      <c r="D13" s="11" t="s">
+      <c r="B13" s="34"/>
+      <c r="D13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="44"/>
-      <c r="G13" s="11" t="s">
+      <c r="E13" s="34"/>
+      <c r="G13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="H13" s="44"/>
-      <c r="J13" s="11" t="s">
+      <c r="H13" s="34"/>
+      <c r="J13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="K13" s="44"/>
+      <c r="K13" s="34"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B14" s="46"/>
-      <c r="D14" s="10" t="s">
+      <c r="B14" s="36"/>
+      <c r="D14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E14" s="46"/>
-      <c r="G14" s="10" t="s">
+      <c r="E14" s="36"/>
+      <c r="G14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H14" s="46"/>
-      <c r="J14" s="10" t="s">
+      <c r="H14" s="36"/>
+      <c r="J14" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="K14" s="46"/>
+      <c r="K14" s="36"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B15" s="47"/>
-      <c r="D15" s="11" t="s">
+      <c r="B15" s="37"/>
+      <c r="D15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="47"/>
-      <c r="G15" s="11" t="s">
+      <c r="E15" s="37"/>
+      <c r="G15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H15" s="47"/>
-      <c r="J15" s="11" t="s">
+      <c r="H15" s="37"/>
+      <c r="J15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K15" s="47"/>
+      <c r="K15" s="37"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="47"/>
-      <c r="D16" s="10" t="s">
+      <c r="B16" s="37"/>
+      <c r="D16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E16" s="47"/>
-      <c r="G16" s="10" t="s">
+      <c r="E16" s="37"/>
+      <c r="G16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H16" s="47"/>
-      <c r="J16" s="10" t="s">
+      <c r="H16" s="37"/>
+      <c r="J16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="K16" s="47"/>
+      <c r="K16" s="37"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="48"/>
-      <c r="D17" s="11" t="s">
+      <c r="B17" s="38"/>
+      <c r="D17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E17" s="48"/>
-      <c r="G17" s="11" t="s">
+      <c r="E17" s="38"/>
+      <c r="G17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H17" s="48"/>
-      <c r="J17" s="11" t="s">
+      <c r="H17" s="38"/>
+      <c r="J17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K17" s="48"/>
+      <c r="K17" s="38"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+      <c r="A18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="48"/>
-      <c r="D18" s="10" t="s">
+      <c r="B18" s="38"/>
+      <c r="D18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E18" s="48"/>
-      <c r="G18" s="10" t="s">
+      <c r="E18" s="38"/>
+      <c r="G18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H18" s="48"/>
-      <c r="J18" s="10" t="s">
+      <c r="H18" s="38"/>
+      <c r="J18" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="K18" s="48"/>
+      <c r="K18" s="38"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B19" s="45"/>
-      <c r="D19" s="11" t="s">
+      <c r="B19" s="35"/>
+      <c r="D19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="E19" s="45"/>
-      <c r="G19" s="11" t="s">
+      <c r="E19" s="35"/>
+      <c r="G19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="H19" s="45"/>
-      <c r="J19" s="11" t="s">
+      <c r="H19" s="35"/>
+      <c r="J19" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="K19" s="45"/>
+      <c r="K19" s="35"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="12"/>
-      <c r="D20" s="13" t="s">
+      <c r="B20" s="3"/>
+      <c r="D20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E20" s="12"/>
-      <c r="G20" s="13" t="s">
+      <c r="E20" s="3"/>
+      <c r="G20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H20" s="12"/>
-      <c r="J20" s="13" t="s">
+      <c r="H20" s="3"/>
+      <c r="J20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="K20" s="12"/>
+      <c r="K20" s="3"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="D21" s="11" t="s">
+      <c r="B21" s="3"/>
+      <c r="D21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="12"/>
-      <c r="G21" s="11" t="s">
+      <c r="E21" s="3"/>
+      <c r="G21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H21" s="12"/>
-      <c r="J21" s="11" t="s">
+      <c r="H21" s="3"/>
+      <c r="J21" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K21" s="12"/>
+      <c r="K21" s="3"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B22" s="12"/>
-      <c r="D22" s="13" t="s">
+      <c r="B22" s="3"/>
+      <c r="D22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E22" s="12"/>
-      <c r="G22" s="13" t="s">
+      <c r="E22" s="3"/>
+      <c r="G22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H22" s="12"/>
-      <c r="J22" s="13" t="s">
+      <c r="H22" s="3"/>
+      <c r="J22" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K22" s="12"/>
+      <c r="K22" s="3"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="45"/>
-      <c r="D23" s="11" t="s">
+      <c r="B23" s="35"/>
+      <c r="D23" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E23" s="45"/>
-      <c r="G23" s="11" t="s">
+      <c r="E23" s="35"/>
+      <c r="G23" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="H23" s="45"/>
-      <c r="J23" s="11" t="s">
+      <c r="H23" s="35"/>
+      <c r="J23" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="K23" s="45"/>
+      <c r="K23" s="35"/>
     </row>
     <row r="25" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="26" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2636,673 +2196,681 @@
   <dimension ref="A1:T51"/>
   <sheetFormatPr defaultColWidth="12.42578125" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17" style="25" customWidth="1"/>
-    <col min="2" max="14" width="12.42578125" style="25"/>
-    <col min="15" max="15" width="21.140625" style="25" customWidth="1"/>
-    <col min="16" max="16384" width="12.42578125" style="25"/>
+    <col min="1" max="1" width="17" style="15" customWidth="1"/>
+    <col min="2" max="14" width="12.42578125" style="15"/>
+    <col min="15" max="15" width="21.140625" style="15" customWidth="1"/>
+    <col min="16" max="16384" width="12.42578125" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
-      <c r="L1" s="22"/>
-      <c r="M1" s="22"/>
-      <c r="N1" s="22"/>
-      <c r="O1" s="23" t="s">
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
+      <c r="G1" s="40"/>
+      <c r="H1" s="40"/>
+      <c r="I1" s="40"/>
+      <c r="J1" s="40"/>
+      <c r="K1" s="40"/>
+      <c r="L1" s="40"/>
+      <c r="M1" s="40"/>
+      <c r="N1" s="40"/>
+      <c r="O1" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="P1" s="24" t="s">
+      <c r="P1" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="24" t="s">
+      <c r="Q1" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="24" t="s">
+      <c r="R1" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="24" t="s">
+      <c r="S1" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="24" t="s">
+      <c r="T1" s="14" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="22"/>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
-      <c r="I2" s="22"/>
-      <c r="J2" s="22"/>
-      <c r="K2" s="22"/>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
-      <c r="N2" s="22"/>
-      <c r="O2" s="26"/>
-      <c r="P2" s="27"/>
-      <c r="Q2" s="27"/>
-      <c r="R2" s="27"/>
-      <c r="S2" s="27"/>
-      <c r="T2" s="27"/>
+      <c r="A2" s="40"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="40"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+      <c r="K2" s="40"/>
+      <c r="L2" s="40"/>
+      <c r="M2" s="40"/>
+      <c r="N2" s="40"/>
+      <c r="O2" s="16"/>
+      <c r="P2" s="17"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
     </row>
     <row r="3" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="22"/>
-      <c r="B3" s="22"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22"/>
-      <c r="I3" s="22"/>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22"/>
-      <c r="L3" s="22"/>
-      <c r="M3" s="22"/>
-      <c r="N3" s="22"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="27"/>
-      <c r="Q3" s="27"/>
-      <c r="R3" s="27"/>
-      <c r="S3" s="27"/>
-      <c r="T3" s="27"/>
+      <c r="A3" s="40"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="40"/>
+      <c r="N3" s="40"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="17"/>
+      <c r="Q3" s="17"/>
+      <c r="R3" s="17"/>
+      <c r="S3" s="17"/>
+      <c r="T3" s="17"/>
     </row>
     <row r="4" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="22"/>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="28"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="27"/>
-      <c r="R4" s="27"/>
-      <c r="S4" s="27"/>
-      <c r="T4" s="27"/>
+      <c r="A4" s="40"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="40"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="40"/>
+      <c r="I4" s="40"/>
+      <c r="J4" s="40"/>
+      <c r="K4" s="40"/>
+      <c r="L4" s="40"/>
+      <c r="M4" s="40"/>
+      <c r="N4" s="40"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
+      <c r="S4" s="17"/>
+      <c r="T4" s="17"/>
     </row>
     <row r="5" spans="1:20" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="O5" s="28"/>
-      <c r="P5" s="27"/>
-      <c r="Q5" s="27"/>
-      <c r="R5" s="27"/>
-      <c r="S5" s="27"/>
-      <c r="T5" s="27"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
+      <c r="R5" s="17"/>
+      <c r="S5" s="17"/>
+      <c r="T5" s="17"/>
     </row>
     <row r="6" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="31"/>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="J6" s="32" t="s">
+      <c r="B6" s="20"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="J6" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="K6" s="33"/>
-      <c r="O6" s="28"/>
-      <c r="P6" s="27"/>
-      <c r="Q6" s="27"/>
-      <c r="R6" s="27"/>
-      <c r="S6" s="27"/>
-      <c r="T6" s="27"/>
+      <c r="K6" s="23"/>
+      <c r="O6" s="18"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
     </row>
     <row r="7" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="34"/>
-      <c r="B7" s="35" t="s">
+      <c r="A7" s="24"/>
+      <c r="B7" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="36"/>
-      <c r="F7" s="36"/>
-      <c r="J7" s="37" t="s">
+      <c r="C7" s="26"/>
+      <c r="D7" s="26"/>
+      <c r="E7" s="26"/>
+      <c r="F7" s="26"/>
+      <c r="J7" s="27" t="s">
         <v>35</v>
       </c>
-      <c r="K7" s="33"/>
-      <c r="O7" s="28"/>
-      <c r="P7" s="27"/>
-      <c r="Q7" s="27"/>
-      <c r="R7" s="27"/>
-      <c r="S7" s="27"/>
-      <c r="T7" s="27"/>
+      <c r="K7" s="23"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="17"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="17"/>
     </row>
     <row r="8" spans="1:20" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="39"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="39"/>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
-      <c r="J8" s="40" t="s">
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="J8" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="K8" s="33"/>
-      <c r="O8" s="28"/>
-      <c r="P8" s="27"/>
-      <c r="Q8" s="27"/>
-      <c r="R8" s="27"/>
-      <c r="S8" s="27"/>
-      <c r="T8" s="27"/>
+      <c r="K8" s="23"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="17"/>
+      <c r="Q8" s="17"/>
+      <c r="R8" s="17"/>
+      <c r="S8" s="17"/>
+      <c r="T8" s="17"/>
     </row>
     <row r="9" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="38" t="s">
+      <c r="A9" s="28" t="s">
         <v>26</v>
       </c>
-      <c r="B9" s="39"/>
-      <c r="C9" s="39"/>
-      <c r="D9" s="39"/>
-      <c r="E9" s="39"/>
-      <c r="F9" s="39"/>
-      <c r="O9" s="28"/>
-      <c r="P9" s="27"/>
-      <c r="Q9" s="27"/>
-      <c r="R9" s="27"/>
-      <c r="S9" s="27"/>
-      <c r="T9" s="27"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="17"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="S9" s="17"/>
+      <c r="T9" s="17"/>
     </row>
     <row r="10" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="38" t="s">
+      <c r="A10" s="28" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="39"/>
-      <c r="C10" s="39"/>
-      <c r="D10" s="39"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="O10" s="28"/>
-      <c r="P10" s="27"/>
-      <c r="Q10" s="27"/>
-      <c r="R10" s="27"/>
-      <c r="S10" s="27"/>
-      <c r="T10" s="27"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="17"/>
+      <c r="Q10" s="17"/>
+      <c r="R10" s="17"/>
+      <c r="S10" s="17"/>
+      <c r="T10" s="17"/>
     </row>
     <row r="11" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="38" t="s">
+      <c r="A11" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="39"/>
-      <c r="C11" s="39"/>
-      <c r="D11" s="39"/>
-      <c r="E11" s="39"/>
-      <c r="F11" s="39"/>
-      <c r="O11" s="28"/>
-      <c r="P11" s="27"/>
-      <c r="Q11" s="27"/>
-      <c r="R11" s="27"/>
-      <c r="S11" s="27"/>
-      <c r="T11" s="27"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="17"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="17"/>
     </row>
     <row r="12" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="38" t="s">
+      <c r="A12" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="39"/>
-      <c r="C12" s="39"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="39"/>
-      <c r="F12" s="39"/>
-      <c r="O12" s="28"/>
-      <c r="P12" s="27"/>
-      <c r="Q12" s="27"/>
-      <c r="R12" s="27"/>
-      <c r="S12" s="27"/>
-      <c r="T12" s="27"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="O12" s="18"/>
+      <c r="P12" s="17"/>
+      <c r="Q12" s="17"/>
+      <c r="R12" s="17"/>
+      <c r="S12" s="17"/>
+      <c r="T12" s="17"/>
     </row>
     <row r="13" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="41" t="s">
+      <c r="A13" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="39"/>
-      <c r="C13" s="39"/>
-      <c r="D13" s="39"/>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="O13" s="28"/>
-      <c r="P13" s="27"/>
-      <c r="Q13" s="27"/>
-      <c r="R13" s="27"/>
-      <c r="S13" s="27"/>
-      <c r="T13" s="27"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="29"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="17"/>
+      <c r="Q13" s="17"/>
+      <c r="R13" s="17"/>
+      <c r="S13" s="17"/>
+      <c r="T13" s="17"/>
     </row>
     <row r="14" spans="1:20" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="O14" s="28"/>
-      <c r="P14" s="27"/>
-      <c r="Q14" s="27"/>
-      <c r="R14" s="27"/>
-      <c r="S14" s="27"/>
-      <c r="T14" s="27"/>
+      <c r="O14" s="18"/>
+      <c r="P14" s="17"/>
+      <c r="Q14" s="17"/>
+      <c r="R14" s="17"/>
+      <c r="S14" s="17"/>
+      <c r="T14" s="17"/>
     </row>
     <row r="15" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="29" t="s">
+      <c r="A15" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="30"/>
-      <c r="C15" s="31"/>
-      <c r="D15" s="31"/>
-      <c r="E15" s="31"/>
-      <c r="F15" s="31"/>
-      <c r="O15" s="28"/>
-      <c r="P15" s="27"/>
-      <c r="Q15" s="27"/>
-      <c r="R15" s="27"/>
-      <c r="S15" s="27"/>
-      <c r="T15" s="27"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="O15" s="18"/>
+      <c r="P15" s="17"/>
+      <c r="Q15" s="17"/>
+      <c r="R15" s="17"/>
+      <c r="S15" s="17"/>
+      <c r="T15" s="17"/>
     </row>
     <row r="16" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
-      <c r="B16" s="34" t="s">
+      <c r="A16" s="24"/>
+      <c r="B16" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="34"/>
-      <c r="E16" s="34"/>
-      <c r="F16" s="34"/>
-      <c r="O16" s="28"/>
-      <c r="P16" s="27"/>
-      <c r="Q16" s="27"/>
-      <c r="R16" s="27"/>
-      <c r="S16" s="27"/>
-      <c r="T16" s="27"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="O16" s="18"/>
+      <c r="P16" s="17"/>
+      <c r="Q16" s="17"/>
+      <c r="R16" s="17"/>
+      <c r="S16" s="17"/>
+      <c r="T16" s="17"/>
     </row>
     <row r="17" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="39"/>
-      <c r="C17" s="39"/>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="O17" s="28"/>
-      <c r="P17" s="27"/>
-      <c r="Q17" s="27"/>
-      <c r="R17" s="27"/>
-      <c r="S17" s="27"/>
-      <c r="T17" s="27"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="29"/>
+      <c r="O17" s="18"/>
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="17"/>
+      <c r="S17" s="17"/>
+      <c r="T17" s="17"/>
     </row>
     <row r="18" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="42" t="s">
+      <c r="A18" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="39"/>
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="O18" s="28"/>
-      <c r="P18" s="27"/>
-      <c r="Q18" s="27"/>
-      <c r="R18" s="27"/>
-      <c r="S18" s="27"/>
-      <c r="T18" s="27"/>
+      <c r="B18" s="29"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="29"/>
+      <c r="O18" s="18"/>
+      <c r="P18" s="17"/>
+      <c r="Q18" s="17"/>
+      <c r="R18" s="17"/>
+      <c r="S18" s="17"/>
+      <c r="T18" s="17"/>
     </row>
     <row r="19" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="42" t="s">
+      <c r="A19" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="39"/>
-      <c r="C19" s="39"/>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="O19" s="28"/>
-      <c r="P19" s="27"/>
-      <c r="Q19" s="27"/>
-      <c r="R19" s="27"/>
-      <c r="S19" s="27"/>
-      <c r="T19" s="27"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="O19" s="18"/>
+      <c r="P19" s="17"/>
+      <c r="Q19" s="17"/>
+      <c r="R19" s="17"/>
+      <c r="S19" s="17"/>
+      <c r="T19" s="17"/>
     </row>
     <row r="20" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="42" t="s">
+      <c r="A20" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="39"/>
-      <c r="C20" s="39"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="O20" s="28"/>
-      <c r="P20" s="27"/>
-      <c r="Q20" s="27"/>
-      <c r="R20" s="27"/>
-      <c r="S20" s="27"/>
-      <c r="T20" s="27"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="O20" s="18"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+      <c r="S20" s="17"/>
+      <c r="T20" s="17"/>
     </row>
     <row r="21" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21"/>
-      <c r="B21"/>
-      <c r="C21"/>
-      <c r="D21"/>
-      <c r="E21"/>
-      <c r="F21"/>
-      <c r="O21" s="28"/>
-      <c r="P21" s="27"/>
-      <c r="Q21" s="27"/>
-      <c r="R21" s="27"/>
-      <c r="S21" s="27"/>
-      <c r="T21" s="27"/>
+      <c r="A21" s="32" t="s">
+        <v>46</v>
+      </c>
+      <c r="B21" s="29"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="29"/>
+      <c r="O21" s="18"/>
+      <c r="P21" s="17"/>
+      <c r="Q21" s="17"/>
+      <c r="R21" s="17"/>
+      <c r="S21" s="17"/>
+      <c r="T21" s="17"/>
     </row>
     <row r="22" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="43" t="s">
-        <v>41</v>
-      </c>
-      <c r="B22" s="43"/>
+      <c r="A22"/>
+      <c r="B22"/>
       <c r="C22"/>
       <c r="D22"/>
       <c r="E22"/>
       <c r="F22"/>
-      <c r="O22" s="28"/>
-      <c r="P22" s="27"/>
-      <c r="Q22" s="27"/>
-      <c r="R22" s="27"/>
-      <c r="S22" s="27"/>
-      <c r="T22" s="27"/>
+      <c r="O22" s="18"/>
+      <c r="P22" s="17"/>
+      <c r="Q22" s="17"/>
+      <c r="R22" s="17"/>
+      <c r="S22" s="17"/>
+      <c r="T22" s="17"/>
     </row>
     <row r="23" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="42" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" s="39"/>
+      <c r="A23" s="33" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" s="33"/>
       <c r="C23"/>
       <c r="D23"/>
       <c r="E23"/>
       <c r="F23"/>
-      <c r="O23" s="28"/>
-      <c r="P23" s="27"/>
-      <c r="Q23" s="27"/>
-      <c r="R23" s="27"/>
-      <c r="S23" s="27"/>
-      <c r="T23" s="27"/>
+      <c r="O23" s="18"/>
+      <c r="P23" s="17"/>
+      <c r="Q23" s="17"/>
+      <c r="R23" s="17"/>
+      <c r="S23" s="17"/>
+      <c r="T23" s="17"/>
     </row>
     <row r="24" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="42" t="s">
-        <v>43</v>
-      </c>
-      <c r="B24" s="39"/>
+      <c r="A24" s="32" t="s">
+        <v>42</v>
+      </c>
+      <c r="B24" s="29"/>
       <c r="C24"/>
       <c r="D24"/>
       <c r="E24"/>
-      <c r="O24" s="28"/>
-      <c r="P24" s="27"/>
-      <c r="Q24" s="27"/>
-      <c r="R24" s="27"/>
-      <c r="S24" s="27"/>
-      <c r="T24" s="27"/>
+      <c r="F24"/>
+      <c r="O24" s="18"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="17"/>
     </row>
     <row r="25" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="B25" s="39"/>
+      <c r="A25" s="32" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" s="29"/>
       <c r="C25"/>
       <c r="D25"/>
       <c r="E25"/>
-      <c r="O25" s="28"/>
-      <c r="P25" s="27"/>
-      <c r="Q25" s="27"/>
-      <c r="R25" s="27"/>
-      <c r="S25" s="27"/>
-      <c r="T25" s="27"/>
-    </row>
-    <row r="26" spans="1:20" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="O26" s="28"/>
-      <c r="P26" s="27"/>
-      <c r="Q26" s="27"/>
-      <c r="R26" s="27"/>
-      <c r="S26" s="27"/>
-      <c r="T26" s="27"/>
-    </row>
-    <row r="27" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="29" t="s">
+      <c r="O25" s="18"/>
+      <c r="P25" s="17"/>
+      <c r="Q25" s="17"/>
+      <c r="R25" s="17"/>
+      <c r="S25" s="17"/>
+      <c r="T25" s="17"/>
+    </row>
+    <row r="26" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="32" t="s">
+        <v>44</v>
+      </c>
+      <c r="B26" s="29"/>
+      <c r="C26"/>
+      <c r="D26"/>
+      <c r="E26"/>
+      <c r="O26" s="18"/>
+      <c r="P26" s="17"/>
+      <c r="Q26" s="17"/>
+      <c r="R26" s="17"/>
+      <c r="S26" s="17"/>
+      <c r="T26" s="17"/>
+    </row>
+    <row r="27" spans="1:20" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="O27" s="18"/>
+      <c r="P27" s="17"/>
+      <c r="Q27" s="17"/>
+      <c r="R27" s="17"/>
+      <c r="S27" s="17"/>
+      <c r="T27" s="17"/>
+    </row>
+    <row r="28" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="30"/>
-      <c r="C27" s="31"/>
-      <c r="D27" s="31"/>
-      <c r="E27" s="31"/>
-      <c r="O27" s="28"/>
-      <c r="P27" s="27"/>
-      <c r="Q27" s="27"/>
-      <c r="R27" s="27"/>
-      <c r="S27" s="27"/>
-      <c r="T27" s="27"/>
-    </row>
-    <row r="28" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="20" t="s">
+      <c r="B28" s="20"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="O28" s="18"/>
+      <c r="P28" s="17"/>
+      <c r="Q28" s="17"/>
+      <c r="R28" s="17"/>
+      <c r="S28" s="17"/>
+      <c r="T28" s="17"/>
+    </row>
+    <row r="29" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B28" s="18"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="19"/>
-      <c r="O28" s="28"/>
-      <c r="P28" s="27"/>
-      <c r="Q28" s="27"/>
-      <c r="R28" s="27"/>
-      <c r="S28" s="27"/>
-      <c r="T28" s="27"/>
-    </row>
-    <row r="29" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="s">
+      <c r="B29" s="9"/>
+      <c r="C29" s="10"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="10"/>
+      <c r="O29" s="18"/>
+      <c r="P29" s="17"/>
+      <c r="Q29" s="17"/>
+      <c r="R29" s="17"/>
+      <c r="S29" s="17"/>
+      <c r="T29" s="17"/>
+    </row>
+    <row r="30" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B29" s="21"/>
-      <c r="C29" s="21"/>
-      <c r="D29" s="21"/>
-      <c r="E29" s="21"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="27"/>
-      <c r="Q29" s="27"/>
-      <c r="R29" s="27"/>
-      <c r="S29" s="27"/>
-      <c r="T29" s="27"/>
-    </row>
-    <row r="30" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O30" s="28"/>
-      <c r="P30" s="27"/>
-      <c r="Q30" s="27"/>
-      <c r="R30" s="27"/>
-      <c r="S30" s="27"/>
-      <c r="T30" s="27"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="O30" s="18"/>
+      <c r="P30" s="17"/>
+      <c r="Q30" s="17"/>
+      <c r="R30" s="17"/>
+      <c r="S30" s="17"/>
+      <c r="T30" s="17"/>
     </row>
     <row r="31" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O31" s="28"/>
-      <c r="P31" s="27"/>
-      <c r="Q31" s="27"/>
-      <c r="R31" s="27"/>
-      <c r="S31" s="27"/>
-      <c r="T31" s="27"/>
+      <c r="O31" s="18"/>
+      <c r="P31" s="17"/>
+      <c r="Q31" s="17"/>
+      <c r="R31" s="17"/>
+      <c r="S31" s="17"/>
+      <c r="T31" s="17"/>
     </row>
     <row r="32" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O32" s="28"/>
-      <c r="P32" s="27"/>
-      <c r="Q32" s="27"/>
-      <c r="R32" s="27"/>
-      <c r="S32" s="27"/>
-      <c r="T32" s="27"/>
+      <c r="O32" s="18"/>
+      <c r="P32" s="17"/>
+      <c r="Q32" s="17"/>
+      <c r="R32" s="17"/>
+      <c r="S32" s="17"/>
+      <c r="T32" s="17"/>
     </row>
     <row r="33" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O33" s="28"/>
-      <c r="P33" s="27"/>
-      <c r="Q33" s="27"/>
-      <c r="R33" s="27"/>
-      <c r="S33" s="27"/>
-      <c r="T33" s="27"/>
+      <c r="O33" s="18"/>
+      <c r="P33" s="17"/>
+      <c r="Q33" s="17"/>
+      <c r="R33" s="17"/>
+      <c r="S33" s="17"/>
+      <c r="T33" s="17"/>
     </row>
     <row r="34" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O34" s="28"/>
-      <c r="P34" s="27"/>
-      <c r="Q34" s="27"/>
-      <c r="R34" s="27"/>
-      <c r="S34" s="27"/>
-      <c r="T34" s="27"/>
+      <c r="O34" s="18"/>
+      <c r="P34" s="17"/>
+      <c r="Q34" s="17"/>
+      <c r="R34" s="17"/>
+      <c r="S34" s="17"/>
+      <c r="T34" s="17"/>
     </row>
     <row r="35" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O35" s="28"/>
-      <c r="P35" s="27"/>
-      <c r="Q35" s="27"/>
-      <c r="R35" s="27"/>
-      <c r="S35" s="27"/>
-      <c r="T35" s="27"/>
+      <c r="O35" s="18"/>
+      <c r="P35" s="17"/>
+      <c r="Q35" s="17"/>
+      <c r="R35" s="17"/>
+      <c r="S35" s="17"/>
+      <c r="T35" s="17"/>
     </row>
     <row r="36" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O36" s="28"/>
-      <c r="P36" s="27"/>
-      <c r="Q36" s="27"/>
-      <c r="R36" s="27"/>
-      <c r="S36" s="27"/>
-      <c r="T36" s="27"/>
+      <c r="O36" s="18"/>
+      <c r="P36" s="17"/>
+      <c r="Q36" s="17"/>
+      <c r="R36" s="17"/>
+      <c r="S36" s="17"/>
+      <c r="T36" s="17"/>
     </row>
     <row r="37" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M37" s="25" t="s">
+      <c r="M37" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="O37" s="28"/>
-      <c r="P37" s="27"/>
-      <c r="Q37" s="27"/>
-      <c r="R37" s="27"/>
-      <c r="S37" s="27"/>
-      <c r="T37" s="27"/>
+      <c r="O37" s="18"/>
+      <c r="P37" s="17"/>
+      <c r="Q37" s="17"/>
+      <c r="R37" s="17"/>
+      <c r="S37" s="17"/>
+      <c r="T37" s="17"/>
     </row>
     <row r="38" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O38" s="28"/>
-      <c r="P38" s="27"/>
-      <c r="Q38" s="27"/>
-      <c r="R38" s="27"/>
-      <c r="S38" s="27"/>
-      <c r="T38" s="27"/>
+      <c r="O38" s="18"/>
+      <c r="P38" s="17"/>
+      <c r="Q38" s="17"/>
+      <c r="R38" s="17"/>
+      <c r="S38" s="17"/>
+      <c r="T38" s="17"/>
     </row>
     <row r="39" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O39" s="28"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="27"/>
-      <c r="S39" s="27"/>
-      <c r="T39" s="27"/>
+      <c r="O39" s="18"/>
+      <c r="P39" s="17"/>
+      <c r="Q39" s="17"/>
+      <c r="R39" s="17"/>
+      <c r="S39" s="17"/>
+      <c r="T39" s="17"/>
     </row>
     <row r="40" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O40" s="28"/>
-      <c r="P40" s="27"/>
-      <c r="Q40" s="27"/>
-      <c r="R40" s="27"/>
-      <c r="S40" s="27"/>
-      <c r="T40" s="27"/>
+      <c r="O40" s="18"/>
+      <c r="P40" s="17"/>
+      <c r="Q40" s="17"/>
+      <c r="R40" s="17"/>
+      <c r="S40" s="17"/>
+      <c r="T40" s="17"/>
     </row>
     <row r="41" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O41" s="28"/>
-      <c r="P41" s="27"/>
-      <c r="Q41" s="27"/>
-      <c r="R41" s="27"/>
-      <c r="S41" s="27"/>
-      <c r="T41" s="27"/>
+      <c r="O41" s="18"/>
+      <c r="P41" s="17"/>
+      <c r="Q41" s="17"/>
+      <c r="R41" s="17"/>
+      <c r="S41" s="17"/>
+      <c r="T41" s="17"/>
     </row>
     <row r="42" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O42" s="28"/>
-      <c r="P42" s="27"/>
-      <c r="Q42" s="27"/>
-      <c r="R42" s="27"/>
-      <c r="S42" s="27"/>
-      <c r="T42" s="27"/>
+      <c r="O42" s="18"/>
+      <c r="P42" s="17"/>
+      <c r="Q42" s="17"/>
+      <c r="R42" s="17"/>
+      <c r="S42" s="17"/>
+      <c r="T42" s="17"/>
     </row>
     <row r="43" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O43" s="28"/>
-      <c r="P43" s="27"/>
-      <c r="Q43" s="27"/>
-      <c r="R43" s="27"/>
-      <c r="S43" s="27"/>
-      <c r="T43" s="27"/>
+      <c r="O43" s="18"/>
+      <c r="P43" s="17"/>
+      <c r="Q43" s="17"/>
+      <c r="R43" s="17"/>
+      <c r="S43" s="17"/>
+      <c r="T43" s="17"/>
     </row>
     <row r="44" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O44" s="28"/>
-      <c r="P44" s="27"/>
-      <c r="Q44" s="27"/>
-      <c r="R44" s="27"/>
-      <c r="S44" s="27"/>
-      <c r="T44" s="27"/>
+      <c r="O44" s="18"/>
+      <c r="P44" s="17"/>
+      <c r="Q44" s="17"/>
+      <c r="R44" s="17"/>
+      <c r="S44" s="17"/>
+      <c r="T44" s="17"/>
     </row>
     <row r="45" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O45" s="28"/>
-      <c r="P45" s="27"/>
-      <c r="Q45" s="27"/>
-      <c r="R45" s="27"/>
-      <c r="S45" s="27"/>
-      <c r="T45" s="27"/>
+      <c r="O45" s="18"/>
+      <c r="P45" s="17"/>
+      <c r="Q45" s="17"/>
+      <c r="R45" s="17"/>
+      <c r="S45" s="17"/>
+      <c r="T45" s="17"/>
     </row>
     <row r="46" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O46" s="28"/>
-      <c r="P46" s="27"/>
-      <c r="Q46" s="27"/>
-      <c r="R46" s="27"/>
-      <c r="S46" s="27"/>
-      <c r="T46" s="27"/>
+      <c r="O46" s="18"/>
+      <c r="P46" s="17"/>
+      <c r="Q46" s="17"/>
+      <c r="R46" s="17"/>
+      <c r="S46" s="17"/>
+      <c r="T46" s="17"/>
     </row>
     <row r="47" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O47" s="28"/>
-      <c r="P47" s="27"/>
-      <c r="Q47" s="27"/>
-      <c r="R47" s="27"/>
-      <c r="S47" s="27"/>
-      <c r="T47" s="27"/>
+      <c r="O47" s="18"/>
+      <c r="P47" s="17"/>
+      <c r="Q47" s="17"/>
+      <c r="R47" s="17"/>
+      <c r="S47" s="17"/>
+      <c r="T47" s="17"/>
     </row>
     <row r="48" spans="13:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O48" s="28"/>
-      <c r="P48" s="27"/>
-      <c r="Q48" s="27"/>
-      <c r="R48" s="27"/>
-      <c r="S48" s="27"/>
-      <c r="T48" s="27"/>
+      <c r="O48" s="18"/>
+      <c r="P48" s="17"/>
+      <c r="Q48" s="17"/>
+      <c r="R48" s="17"/>
+      <c r="S48" s="17"/>
+      <c r="T48" s="17"/>
     </row>
     <row r="49" spans="15:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O49" s="28"/>
-      <c r="P49" s="27"/>
-      <c r="Q49" s="27"/>
-      <c r="R49" s="27"/>
-      <c r="S49" s="27"/>
-      <c r="T49" s="27"/>
+      <c r="O49" s="18"/>
+      <c r="P49" s="17"/>
+      <c r="Q49" s="17"/>
+      <c r="R49" s="17"/>
+      <c r="S49" s="17"/>
+      <c r="T49" s="17"/>
     </row>
     <row r="50" spans="15:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O50" s="28"/>
-      <c r="P50" s="27"/>
-      <c r="Q50" s="27"/>
-      <c r="R50" s="27"/>
-      <c r="S50" s="27"/>
-      <c r="T50" s="27"/>
+      <c r="O50" s="18"/>
+      <c r="P50" s="17"/>
+      <c r="Q50" s="17"/>
+      <c r="R50" s="17"/>
+      <c r="S50" s="17"/>
+      <c r="T50" s="17"/>
     </row>
     <row r="51" spans="15:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="O51" s="28"/>
-      <c r="P51" s="27"/>
-      <c r="Q51" s="27"/>
-      <c r="R51" s="27"/>
-      <c r="S51" s="27"/>
-      <c r="T51" s="27"/>
+      <c r="O51" s="18"/>
+      <c r="P51" s="17"/>
+      <c r="Q51" s="17"/>
+      <c r="R51" s="17"/>
+      <c r="S51" s="17"/>
+      <c r="T51" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>